<commit_message>
Final compliance audit and Excel pilot matrix standardization. All services now routing and quoting correctly as per pricing sheet.
</commit_message>
<xml_diff>
--- a/DIFM_Pilot_Matrix_v1_Baseline.xlsx
+++ b/DIFM_Pilot_Matrix_v1_Baseline.xlsx
@@ -522,13 +522,13 @@
         <v>risk_class</v>
       </c>
       <c r="N1" t="str">
+        <v>admin_review_required</v>
+      </c>
+      <c r="O1" t="str">
         <v>evidence_override</v>
       </c>
-      <c r="O1" t="str">
+      <c r="P1" t="str">
         <v>scope_guard_group</v>
-      </c>
-      <c r="P1" t="str">
-        <v>admin_review_required</v>
       </c>
     </row>
     <row r="2">
@@ -571,7 +571,7 @@
       <c r="M2" t="str">
         <v>LOW</v>
       </c>
-      <c r="P2" t="str">
+      <c r="N2" t="str">
         <v>Y</v>
       </c>
     </row>
@@ -609,7 +609,7 @@
       <c r="M3" t="str">
         <v>LOW</v>
       </c>
-      <c r="P3" t="str">
+      <c r="N3" t="str">
         <v>Y</v>
       </c>
     </row>
@@ -647,7 +647,7 @@
       <c r="M4" t="str">
         <v>LOW</v>
       </c>
-      <c r="P4" t="str">
+      <c r="N4" t="str">
         <v>Y</v>
       </c>
     </row>
@@ -686,13 +686,13 @@
         <v>LOW</v>
       </c>
       <c r="N5" t="str">
+        <v>N</v>
+      </c>
+      <c r="O5" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O5" t="str">
+      <c r="P5" t="str">
         <v>DRILLING</v>
-      </c>
-      <c r="P5" t="str">
-        <v>N</v>
       </c>
     </row>
     <row r="6">
@@ -733,13 +733,13 @@
         <v>LOW</v>
       </c>
       <c r="N6" t="str">
+        <v>Y</v>
+      </c>
+      <c r="O6" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O6" t="str">
+      <c r="P6" t="str">
         <v>PLUMBING_RISK</v>
-      </c>
-      <c r="P6" t="str">
-        <v>Y</v>
       </c>
     </row>
     <row r="7">
@@ -779,7 +779,7 @@
       <c r="M7" t="str">
         <v>HIGH_RISK</v>
       </c>
-      <c r="P7" t="str">
+      <c r="N7" t="str">
         <v>Y</v>
       </c>
     </row>
@@ -817,7 +817,7 @@
       <c r="M8" t="str">
         <v>LOW</v>
       </c>
-      <c r="P8" t="str">
+      <c r="N8" t="str">
         <v>N</v>
       </c>
     </row>
@@ -832,7 +832,7 @@
         <v>HANDYMAN</v>
       </c>
       <c r="D9">
-        <v>75</v>
+        <v>60</v>
       </c>
       <c r="E9" t="str">
         <v>N</v>
@@ -856,13 +856,13 @@
         <v>LOW</v>
       </c>
       <c r="N9" t="str">
+        <v>Y</v>
+      </c>
+      <c r="O9" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O9" t="str">
+      <c r="P9" t="str">
         <v>DRILLING</v>
-      </c>
-      <c r="P9" t="str">
-        <v>Y</v>
       </c>
     </row>
     <row r="10">
@@ -899,7 +899,7 @@
       <c r="M10" t="str">
         <v>LOW</v>
       </c>
-      <c r="P10" t="str">
+      <c r="N10" t="str">
         <v>N</v>
       </c>
     </row>
@@ -937,7 +937,7 @@
       <c r="M11" t="str">
         <v>LOW</v>
       </c>
-      <c r="P11" t="str">
+      <c r="N11" t="str">
         <v>N</v>
       </c>
     </row>
@@ -976,13 +976,13 @@
         <v>LOW</v>
       </c>
       <c r="N12" t="str">
+        <v>N</v>
+      </c>
+      <c r="O12" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O12" t="str">
+      <c r="P12" t="str">
         <v>DRILLING</v>
-      </c>
-      <c r="P12" t="str">
-        <v>N</v>
       </c>
     </row>
     <row r="13">
@@ -996,7 +996,7 @@
         <v>HANDYMAN</v>
       </c>
       <c r="D13">
-        <v>75</v>
+        <v>60</v>
       </c>
       <c r="E13" t="str">
         <v>N</v>
@@ -1020,13 +1020,13 @@
         <v>LOW</v>
       </c>
       <c r="N13" t="str">
+        <v>Y</v>
+      </c>
+      <c r="O13" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O13" t="str">
+      <c r="P13" t="str">
         <v>DRILLING</v>
-      </c>
-      <c r="P13" t="str">
-        <v>Y</v>
       </c>
     </row>
     <row r="14">
@@ -1040,7 +1040,7 @@
         <v>ELECTRICAL</v>
       </c>
       <c r="D14">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="E14" t="str">
         <v>Y</v>
@@ -1067,13 +1067,13 @@
         <v>HIGH_RISK</v>
       </c>
       <c r="N14" t="str">
+        <v>Y</v>
+      </c>
+      <c r="O14" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O14" t="str">
+      <c r="P14" t="str">
         <v>ELECTRICAL_RISK</v>
-      </c>
-      <c r="P14" t="str">
-        <v>Y</v>
       </c>
     </row>
     <row r="15">
@@ -1087,7 +1087,7 @@
         <v>PLUMBING</v>
       </c>
       <c r="D15">
-        <v>75</v>
+        <v>60</v>
       </c>
       <c r="E15" t="str">
         <v>N</v>
@@ -1111,13 +1111,13 @@
         <v>HIGH_RISK</v>
       </c>
       <c r="N15" t="str">
+        <v>Y</v>
+      </c>
+      <c r="O15" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O15" t="str">
+      <c r="P15" t="str">
         <v>PLUMBING_RISK</v>
-      </c>
-      <c r="P15" t="str">
-        <v>Y</v>
       </c>
     </row>
     <row r="16">
@@ -1155,13 +1155,13 @@
         <v>LOW</v>
       </c>
       <c r="N16" t="str">
+        <v>Y</v>
+      </c>
+      <c r="O16" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O16" t="str">
+      <c r="P16" t="str">
         <v>PLUMBING_RISK</v>
-      </c>
-      <c r="P16" t="str">
-        <v>Y</v>
       </c>
     </row>
     <row r="17">
@@ -1175,7 +1175,7 @@
         <v>HANDYMAN</v>
       </c>
       <c r="D17">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="E17" t="str">
         <v>Y</v>
@@ -1205,13 +1205,13 @@
         <v>LOW</v>
       </c>
       <c r="N17" t="str">
+        <v>Y</v>
+      </c>
+      <c r="O17" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O17" t="str">
+      <c r="P17" t="str">
         <v>DRILLING</v>
-      </c>
-      <c r="P17" t="str">
-        <v>Y</v>
       </c>
     </row>
     <row r="18">
@@ -1252,13 +1252,13 @@
         <v>LOW</v>
       </c>
       <c r="N18" t="str">
+        <v>N</v>
+      </c>
+      <c r="O18" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O18" t="str">
+      <c r="P18" t="str">
         <v>ELECTRICAL_RISK</v>
-      </c>
-      <c r="P18" t="str">
-        <v>N</v>
       </c>
     </row>
     <row r="19">
@@ -1298,7 +1298,7 @@
       <c r="M19" t="str">
         <v>LOW</v>
       </c>
-      <c r="P19" t="str">
+      <c r="N19" t="str">
         <v>N</v>
       </c>
     </row>
@@ -1339,7 +1339,7 @@
       <c r="M20" t="str">
         <v>LOW</v>
       </c>
-      <c r="P20" t="str">
+      <c r="N20" t="str">
         <v>N</v>
       </c>
     </row>
@@ -1380,7 +1380,7 @@
       <c r="M21" t="str">
         <v>LOW</v>
       </c>
-      <c r="P21" t="str">
+      <c r="N21" t="str">
         <v>N</v>
       </c>
     </row>
@@ -1422,13 +1422,13 @@
         <v>LOW</v>
       </c>
       <c r="N22" t="str">
+        <v>N</v>
+      </c>
+      <c r="O22" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O22" t="str">
+      <c r="P22" t="str">
         <v>DRILLING</v>
-      </c>
-      <c r="P22" t="str">
-        <v>N</v>
       </c>
     </row>
     <row r="23">
@@ -1469,13 +1469,13 @@
         <v>LOW</v>
       </c>
       <c r="N23" t="str">
+        <v>N</v>
+      </c>
+      <c r="O23" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O23" t="str">
+      <c r="P23" t="str">
         <v>DRILLING</v>
-      </c>
-      <c r="P23" t="str">
-        <v>N</v>
       </c>
     </row>
     <row r="24">
@@ -1515,7 +1515,7 @@
       <c r="M24" t="str">
         <v>LOW</v>
       </c>
-      <c r="P24" t="str">
+      <c r="N24" t="str">
         <v>N</v>
       </c>
     </row>
@@ -1557,13 +1557,13 @@
         <v>LOW</v>
       </c>
       <c r="N25" t="str">
+        <v>N</v>
+      </c>
+      <c r="O25" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O25" t="str">
+      <c r="P25" t="str">
         <v>DRILLING</v>
-      </c>
-      <c r="P25" t="str">
-        <v>N</v>
       </c>
     </row>
     <row r="26">
@@ -1604,13 +1604,13 @@
         <v>LOW</v>
       </c>
       <c r="N26" t="str">
+        <v>N</v>
+      </c>
+      <c r="O26" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O26" t="str">
+      <c r="P26" t="str">
         <v>DRILLING</v>
-      </c>
-      <c r="P26" t="str">
-        <v>N</v>
       </c>
     </row>
     <row r="27">
@@ -1651,13 +1651,13 @@
         <v>LOW</v>
       </c>
       <c r="N27" t="str">
+        <v>N</v>
+      </c>
+      <c r="O27" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O27" t="str">
+      <c r="P27" t="str">
         <v>DRILLING</v>
-      </c>
-      <c r="P27" t="str">
-        <v>N</v>
       </c>
     </row>
     <row r="28">
@@ -1698,13 +1698,13 @@
         <v>LOW</v>
       </c>
       <c r="N28" t="str">
+        <v>N</v>
+      </c>
+      <c r="O28" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O28" t="str">
+      <c r="P28" t="str">
         <v>PLUMBING_RISK</v>
-      </c>
-      <c r="P28" t="str">
-        <v>N</v>
       </c>
     </row>
     <row r="29">
@@ -1744,7 +1744,7 @@
       <c r="M29" t="str">
         <v>LOW</v>
       </c>
-      <c r="P29" t="str">
+      <c r="N29" t="str">
         <v>N</v>
       </c>
     </row>
@@ -1786,13 +1786,13 @@
         <v>LOW</v>
       </c>
       <c r="N30" t="str">
+        <v>N</v>
+      </c>
+      <c r="O30" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O30" t="str">
+      <c r="P30" t="str">
         <v>DRILLING</v>
-      </c>
-      <c r="P30" t="str">
-        <v>N</v>
       </c>
     </row>
     <row r="31">
@@ -1832,7 +1832,7 @@
       <c r="M31" t="str">
         <v>LOW</v>
       </c>
-      <c r="P31" t="str">
+      <c r="N31" t="str">
         <v>N</v>
       </c>
     </row>
@@ -1873,7 +1873,7 @@
       <c r="M32" t="str">
         <v>LOW</v>
       </c>
-      <c r="P32" t="str">
+      <c r="N32" t="str">
         <v>N</v>
       </c>
     </row>
@@ -1915,13 +1915,13 @@
         <v>LOW</v>
       </c>
       <c r="N33" t="str">
+        <v>N</v>
+      </c>
+      <c r="O33" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O33" t="str">
+      <c r="P33" t="str">
         <v>DRILLING</v>
-      </c>
-      <c r="P33" t="str">
-        <v>N</v>
       </c>
     </row>
     <row r="34">
@@ -1961,7 +1961,7 @@
       <c r="M34" t="str">
         <v>LOW</v>
       </c>
-      <c r="P34" t="str">
+      <c r="N34" t="str">
         <v>N</v>
       </c>
     </row>
@@ -2003,13 +2003,13 @@
         <v>LOW</v>
       </c>
       <c r="N35" t="str">
+        <v>N</v>
+      </c>
+      <c r="O35" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O35" t="str">
+      <c r="P35" t="str">
         <v>DRILLING</v>
-      </c>
-      <c r="P35" t="str">
-        <v>N</v>
       </c>
     </row>
     <row r="36">
@@ -2050,13 +2050,13 @@
         <v>LOW</v>
       </c>
       <c r="N36" t="str">
+        <v>N</v>
+      </c>
+      <c r="O36" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O36" t="str">
+      <c r="P36" t="str">
         <v>DRILLING</v>
-      </c>
-      <c r="P36" t="str">
-        <v>N</v>
       </c>
     </row>
     <row r="37">
@@ -2097,13 +2097,13 @@
         <v>LOW</v>
       </c>
       <c r="N37" t="str">
+        <v>N</v>
+      </c>
+      <c r="O37" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O37" t="str">
+      <c r="P37" t="str">
         <v>DRILLING</v>
-      </c>
-      <c r="P37" t="str">
-        <v>N</v>
       </c>
     </row>
     <row r="38">
@@ -2144,13 +2144,13 @@
         <v>LOW</v>
       </c>
       <c r="N38" t="str">
+        <v>N</v>
+      </c>
+      <c r="O38" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O38" t="str">
+      <c r="P38" t="str">
         <v>DRILLING</v>
-      </c>
-      <c r="P38" t="str">
-        <v>N</v>
       </c>
     </row>
     <row r="39">
@@ -2191,13 +2191,13 @@
         <v>LOW</v>
       </c>
       <c r="N39" t="str">
+        <v>N</v>
+      </c>
+      <c r="O39" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O39" t="str">
+      <c r="P39" t="str">
         <v>DRILLING</v>
-      </c>
-      <c r="P39" t="str">
-        <v>N</v>
       </c>
     </row>
     <row r="40">
@@ -2238,13 +2238,13 @@
         <v>LOW</v>
       </c>
       <c r="N40" t="str">
+        <v>N</v>
+      </c>
+      <c r="O40" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O40" t="str">
+      <c r="P40" t="str">
         <v>DRILLING</v>
-      </c>
-      <c r="P40" t="str">
-        <v>N</v>
       </c>
     </row>
     <row r="41">
@@ -2284,7 +2284,7 @@
       <c r="M41" t="str">
         <v>LOW</v>
       </c>
-      <c r="P41" t="str">
+      <c r="N41" t="str">
         <v>N</v>
       </c>
     </row>
@@ -2326,13 +2326,13 @@
         <v>LOW</v>
       </c>
       <c r="N42" t="str">
+        <v>N</v>
+      </c>
+      <c r="O42" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O42" t="str">
+      <c r="P42" t="str">
         <v>DRILLING</v>
-      </c>
-      <c r="P42" t="str">
-        <v>N</v>
       </c>
     </row>
     <row r="43">
@@ -2373,13 +2373,13 @@
         <v>LOW</v>
       </c>
       <c r="N43" t="str">
+        <v>N</v>
+      </c>
+      <c r="O43" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O43" t="str">
+      <c r="P43" t="str">
         <v>PLUMBING_RISK</v>
-      </c>
-      <c r="P43" t="str">
-        <v>N</v>
       </c>
     </row>
     <row r="44">
@@ -2420,13 +2420,13 @@
         <v>LOW</v>
       </c>
       <c r="N44" t="str">
+        <v>N</v>
+      </c>
+      <c r="O44" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O44" t="str">
+      <c r="P44" t="str">
         <v>PLUMBING_RISK</v>
-      </c>
-      <c r="P44" t="str">
-        <v>N</v>
       </c>
     </row>
     <row r="45">
@@ -2467,13 +2467,13 @@
         <v>LOW</v>
       </c>
       <c r="N45" t="str">
+        <v>N</v>
+      </c>
+      <c r="O45" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O45" t="str">
+      <c r="P45" t="str">
         <v>PLUMBING_RISK</v>
-      </c>
-      <c r="P45" t="str">
-        <v>N</v>
       </c>
     </row>
     <row r="46">
@@ -2513,7 +2513,7 @@
       <c r="M46" t="str">
         <v>LOW</v>
       </c>
-      <c r="P46" t="str">
+      <c r="N46" t="str">
         <v>N</v>
       </c>
     </row>
@@ -2555,13 +2555,13 @@
         <v>LOW</v>
       </c>
       <c r="N47" t="str">
+        <v>N</v>
+      </c>
+      <c r="O47" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O47" t="str">
+      <c r="P47" t="str">
         <v>PLUMBING_RISK</v>
-      </c>
-      <c r="P47" t="str">
-        <v>N</v>
       </c>
     </row>
     <row r="48">
@@ -2602,13 +2602,13 @@
         <v>LOW</v>
       </c>
       <c r="N48" t="str">
+        <v>N</v>
+      </c>
+      <c r="O48" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O48" t="str">
+      <c r="P48" t="str">
         <v>PLUMBING_RISK</v>
-      </c>
-      <c r="P48" t="str">
-        <v>N</v>
       </c>
     </row>
     <row r="49">
@@ -2649,13 +2649,13 @@
         <v>LOW</v>
       </c>
       <c r="N49" t="str">
+        <v>N</v>
+      </c>
+      <c r="O49" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O49" t="str">
+      <c r="P49" t="str">
         <v>PLUMBING_RISK</v>
-      </c>
-      <c r="P49" t="str">
-        <v>N</v>
       </c>
     </row>
     <row r="50">
@@ -2699,13 +2699,13 @@
         <v>LOW</v>
       </c>
       <c r="N50" t="str">
+        <v>Y</v>
+      </c>
+      <c r="O50" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O50" t="str">
+      <c r="P50" t="str">
         <v>DRILLING</v>
-      </c>
-      <c r="P50" t="str">
-        <v>Y</v>
       </c>
     </row>
     <row r="51">
@@ -2746,13 +2746,13 @@
         <v>HIGH_RISK</v>
       </c>
       <c r="N51" t="str">
+        <v>Y</v>
+      </c>
+      <c r="O51" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O51" t="str">
+      <c r="P51" t="str">
         <v>PLUMBING_RISK</v>
-      </c>
-      <c r="P51" t="str">
-        <v>Y</v>
       </c>
     </row>
     <row r="52">
@@ -2793,13 +2793,13 @@
         <v>LOW</v>
       </c>
       <c r="N52" t="str">
+        <v>N</v>
+      </c>
+      <c r="O52" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O52" t="str">
+      <c r="P52" t="str">
         <v>PLUMBING_RISK</v>
-      </c>
-      <c r="P52" t="str">
-        <v>N</v>
       </c>
     </row>
     <row r="53">
@@ -2839,7 +2839,7 @@
       <c r="M53" t="str">
         <v>LOW</v>
       </c>
-      <c r="P53" t="str">
+      <c r="N53" t="str">
         <v>N</v>
       </c>
     </row>
@@ -2881,13 +2881,13 @@
         <v>HIGH_RISK</v>
       </c>
       <c r="N54" t="str">
+        <v>Y</v>
+      </c>
+      <c r="O54" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O54" t="str">
+      <c r="P54" t="str">
         <v>PLUMBING_RISK</v>
-      </c>
-      <c r="P54" t="str">
-        <v>Y</v>
       </c>
     </row>
     <row r="55">
@@ -2928,13 +2928,13 @@
         <v>LOW</v>
       </c>
       <c r="N55" t="str">
+        <v>N</v>
+      </c>
+      <c r="O55" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O55" t="str">
+      <c r="P55" t="str">
         <v>ELECTRICAL_RISK</v>
-      </c>
-      <c r="P55" t="str">
-        <v>N</v>
       </c>
     </row>
     <row r="56">
@@ -2975,13 +2975,13 @@
         <v>LOW</v>
       </c>
       <c r="N56" t="str">
+        <v>Y</v>
+      </c>
+      <c r="O56" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O56" t="str">
+      <c r="P56" t="str">
         <v>ELECTRICAL_RISK</v>
-      </c>
-      <c r="P56" t="str">
-        <v>Y</v>
       </c>
     </row>
     <row r="57">
@@ -3022,13 +3022,13 @@
         <v>LOW</v>
       </c>
       <c r="N57" t="str">
+        <v>N</v>
+      </c>
+      <c r="O57" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O57" t="str">
+      <c r="P57" t="str">
         <v>ELECTRICAL_RISK</v>
-      </c>
-      <c r="P57" t="str">
-        <v>N</v>
       </c>
     </row>
     <row r="58">
@@ -3069,13 +3069,13 @@
         <v>HIGH_RISK</v>
       </c>
       <c r="N58" t="str">
+        <v>Y</v>
+      </c>
+      <c r="O58" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O58" t="str">
+      <c r="P58" t="str">
         <v>ELECTRICAL_RISK</v>
-      </c>
-      <c r="P58" t="str">
-        <v>Y</v>
       </c>
     </row>
     <row r="59">
@@ -3116,13 +3116,13 @@
         <v>HIGH_RISK</v>
       </c>
       <c r="N59" t="str">
+        <v>Y</v>
+      </c>
+      <c r="O59" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O59" t="str">
+      <c r="P59" t="str">
         <v>PLUMBING_RISK</v>
-      </c>
-      <c r="P59" t="str">
-        <v>Y</v>
       </c>
     </row>
     <row r="60">
@@ -3163,13 +3163,13 @@
         <v>HIGH_RISK</v>
       </c>
       <c r="N60" t="str">
+        <v>Y</v>
+      </c>
+      <c r="O60" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O60" t="str">
+      <c r="P60" t="str">
         <v>ELECTRICAL_RISK</v>
-      </c>
-      <c r="P60" t="str">
-        <v>Y</v>
       </c>
     </row>
     <row r="61">
@@ -3209,7 +3209,7 @@
       <c r="M61" t="str">
         <v>LOW</v>
       </c>
-      <c r="P61" t="str">
+      <c r="N61" t="str">
         <v>Y</v>
       </c>
     </row>
@@ -3250,7 +3250,7 @@
       <c r="M62" t="str">
         <v>LOW</v>
       </c>
-      <c r="P62" t="str">
+      <c r="N62" t="str">
         <v>N</v>
       </c>
     </row>
@@ -3291,7 +3291,7 @@
       <c r="M63" t="str">
         <v>LOW</v>
       </c>
-      <c r="P63" t="str">
+      <c r="N63" t="str">
         <v>N</v>
       </c>
     </row>
@@ -3333,13 +3333,13 @@
         <v>LOW</v>
       </c>
       <c r="N64" t="str">
+        <v>Y</v>
+      </c>
+      <c r="O64" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O64" t="str">
+      <c r="P64" t="str">
         <v>PLUMBING_RISK</v>
-      </c>
-      <c r="P64" t="str">
-        <v>Y</v>
       </c>
     </row>
     <row r="65">
@@ -3380,13 +3380,13 @@
         <v>LOW</v>
       </c>
       <c r="N65" t="str">
+        <v>Y</v>
+      </c>
+      <c r="O65" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O65" t="str">
+      <c r="P65" t="str">
         <v>PLUMBING_RISK</v>
-      </c>
-      <c r="P65" t="str">
-        <v>Y</v>
       </c>
     </row>
     <row r="66">
@@ -3427,13 +3427,13 @@
         <v>LOW</v>
       </c>
       <c r="N66" t="str">
+        <v>Y</v>
+      </c>
+      <c r="O66" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O66" t="str">
+      <c r="P66" t="str">
         <v>PLUMBING_RISK</v>
-      </c>
-      <c r="P66" t="str">
-        <v>Y</v>
       </c>
     </row>
     <row r="67">
@@ -3474,13 +3474,13 @@
         <v>LOW</v>
       </c>
       <c r="N67" t="str">
+        <v>Y</v>
+      </c>
+      <c r="O67" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O67" t="str">
+      <c r="P67" t="str">
         <v>PLUMBING_RISK</v>
-      </c>
-      <c r="P67" t="str">
-        <v>Y</v>
       </c>
     </row>
     <row r="68">
@@ -3521,13 +3521,13 @@
         <v>LOW</v>
       </c>
       <c r="N68" t="str">
+        <v>Y</v>
+      </c>
+      <c r="O68" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O68" t="str">
+      <c r="P68" t="str">
         <v>PLUMBING_RISK</v>
-      </c>
-      <c r="P68" t="str">
-        <v>Y</v>
       </c>
     </row>
     <row r="69">
@@ -3567,7 +3567,7 @@
       <c r="M69" t="str">
         <v>LOW</v>
       </c>
-      <c r="P69" t="str">
+      <c r="N69" t="str">
         <v>Y</v>
       </c>
     </row>
@@ -3608,7 +3608,7 @@
       <c r="M70" t="str">
         <v>LOW</v>
       </c>
-      <c r="P70" t="str">
+      <c r="N70" t="str">
         <v>Y</v>
       </c>
     </row>
@@ -3649,7 +3649,7 @@
       <c r="M71" t="str">
         <v>LOW</v>
       </c>
-      <c r="P71" t="str">
+      <c r="N71" t="str">
         <v>Y</v>
       </c>
     </row>
@@ -3690,7 +3690,7 @@
       <c r="M72" t="str">
         <v>LOW</v>
       </c>
-      <c r="P72" t="str">
+      <c r="N72" t="str">
         <v>Y</v>
       </c>
     </row>
@@ -3732,13 +3732,13 @@
         <v>LOW</v>
       </c>
       <c r="N73" t="str">
+        <v>N</v>
+      </c>
+      <c r="O73" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O73" t="str">
+      <c r="P73" t="str">
         <v>DRILLING</v>
-      </c>
-      <c r="P73" t="str">
-        <v>N</v>
       </c>
     </row>
     <row r="74">
@@ -3778,7 +3778,7 @@
       <c r="M74" t="str">
         <v>LOW</v>
       </c>
-      <c r="P74" t="str">
+      <c r="N74" t="str">
         <v>N</v>
       </c>
     </row>
@@ -3819,7 +3819,7 @@
       <c r="M75" t="str">
         <v>LOW</v>
       </c>
-      <c r="P75" t="str">
+      <c r="N75" t="str">
         <v>N</v>
       </c>
     </row>
@@ -3861,13 +3861,13 @@
         <v>LOW</v>
       </c>
       <c r="N76" t="str">
+        <v>N</v>
+      </c>
+      <c r="O76" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O76" t="str">
+      <c r="P76" t="str">
         <v>DRILLING</v>
-      </c>
-      <c r="P76" t="str">
-        <v>N</v>
       </c>
     </row>
     <row r="77">
@@ -3908,13 +3908,13 @@
         <v>LOW</v>
       </c>
       <c r="N77" t="str">
+        <v>N</v>
+      </c>
+      <c r="O77" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O77" t="str">
+      <c r="P77" t="str">
         <v>DRILLING</v>
-      </c>
-      <c r="P77" t="str">
-        <v>N</v>
       </c>
     </row>
     <row r="78">
@@ -3955,13 +3955,13 @@
         <v>LOW</v>
       </c>
       <c r="N78" t="str">
+        <v>N</v>
+      </c>
+      <c r="O78" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O78" t="str">
+      <c r="P78" t="str">
         <v>DRILLING</v>
-      </c>
-      <c r="P78" t="str">
-        <v>N</v>
       </c>
     </row>
     <row r="79">
@@ -4001,7 +4001,7 @@
       <c r="M79" t="str">
         <v>LOW</v>
       </c>
-      <c r="P79" t="str">
+      <c r="N79" t="str">
         <v>N</v>
       </c>
     </row>
@@ -4043,13 +4043,13 @@
         <v>LOW</v>
       </c>
       <c r="N80" t="str">
+        <v>N</v>
+      </c>
+      <c r="O80" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O80" t="str">
+      <c r="P80" t="str">
         <v>PLUMBING_RISK</v>
-      </c>
-      <c r="P80" t="str">
-        <v>N</v>
       </c>
     </row>
     <row r="81">
@@ -4090,13 +4090,13 @@
         <v>LOW</v>
       </c>
       <c r="N81" t="str">
+        <v>N</v>
+      </c>
+      <c r="O81" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O81" t="str">
+      <c r="P81" t="str">
         <v>DRILLING</v>
-      </c>
-      <c r="P81" t="str">
-        <v>N</v>
       </c>
     </row>
     <row r="82">
@@ -4137,13 +4137,13 @@
         <v>LOW</v>
       </c>
       <c r="N82" t="str">
+        <v>N</v>
+      </c>
+      <c r="O82" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O82" t="str">
+      <c r="P82" t="str">
         <v>DRILLING</v>
-      </c>
-      <c r="P82" t="str">
-        <v>N</v>
       </c>
     </row>
     <row r="83">
@@ -4186,7 +4186,7 @@
       <c r="M83" t="str">
         <v>LOW</v>
       </c>
-      <c r="P83" t="str">
+      <c r="N83" t="str">
         <v>N</v>
       </c>
     </row>
@@ -4231,13 +4231,13 @@
         <v>LOW</v>
       </c>
       <c r="N84" t="str">
+        <v>N</v>
+      </c>
+      <c r="O84" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O84" t="str">
+      <c r="P84" t="str">
         <v>DRILLING</v>
-      </c>
-      <c r="P84" t="str">
-        <v>N</v>
       </c>
     </row>
     <row r="85">
@@ -4280,7 +4280,7 @@
       <c r="M85" t="str">
         <v>LOW</v>
       </c>
-      <c r="P85" t="str">
+      <c r="N85" t="str">
         <v>N</v>
       </c>
     </row>
@@ -4324,7 +4324,7 @@
       <c r="M86" t="str">
         <v>LOW</v>
       </c>
-      <c r="P86" t="str">
+      <c r="N86" t="str">
         <v>N</v>
       </c>
     </row>
@@ -4369,13 +4369,13 @@
         <v>LOW</v>
       </c>
       <c r="N87" t="str">
+        <v>N</v>
+      </c>
+      <c r="O87" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O87" t="str">
+      <c r="P87" t="str">
         <v>PLUMBING_RISK</v>
-      </c>
-      <c r="P87" t="str">
-        <v>N</v>
       </c>
     </row>
     <row r="88">
@@ -4418,7 +4418,7 @@
       <c r="M88" t="str">
         <v>LOW</v>
       </c>
-      <c r="P88" t="str">
+      <c r="N88" t="str">
         <v>N</v>
       </c>
     </row>
@@ -4462,7 +4462,7 @@
       <c r="M89" t="str">
         <v>LOW</v>
       </c>
-      <c r="P89" t="str">
+      <c r="N89" t="str">
         <v>N</v>
       </c>
     </row>
@@ -4507,13 +4507,13 @@
         <v>HIGH_RISK</v>
       </c>
       <c r="N90" t="str">
+        <v>N</v>
+      </c>
+      <c r="O90" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O90" t="str">
+      <c r="P90" t="str">
         <v>PLUMBING_RISK</v>
-      </c>
-      <c r="P90" t="str">
-        <v>N</v>
       </c>
     </row>
     <row r="91">
@@ -4557,13 +4557,13 @@
         <v>HIGH_RISK</v>
       </c>
       <c r="N91" t="str">
+        <v>N</v>
+      </c>
+      <c r="O91" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O91" t="str">
+      <c r="P91" t="str">
         <v>PLUMBING_RISK</v>
-      </c>
-      <c r="P91" t="str">
-        <v>N</v>
       </c>
     </row>
     <row r="92">
@@ -4607,13 +4607,13 @@
         <v>HIGH_RISK</v>
       </c>
       <c r="N92" t="str">
+        <v>N</v>
+      </c>
+      <c r="O92" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O92" t="str">
+      <c r="P92" t="str">
         <v>ELECTRICAL_RISK</v>
-      </c>
-      <c r="P92" t="str">
-        <v>N</v>
       </c>
     </row>
     <row r="93">
@@ -4657,13 +4657,13 @@
         <v>HIGH_RISK</v>
       </c>
       <c r="N93" t="str">
+        <v>N</v>
+      </c>
+      <c r="O93" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O93" t="str">
+      <c r="P93" t="str">
         <v>ELECTRICAL_RISK</v>
-      </c>
-      <c r="P93" t="str">
-        <v>N</v>
       </c>
     </row>
     <row r="94">
@@ -4706,7 +4706,7 @@
       <c r="M94" t="str">
         <v>LOW</v>
       </c>
-      <c r="P94" t="str">
+      <c r="N94" t="str">
         <v>N</v>
       </c>
     </row>
@@ -4750,7 +4750,7 @@
       <c r="M95" t="str">
         <v>LOW</v>
       </c>
-      <c r="P95" t="str">
+      <c r="N95" t="str">
         <v>N</v>
       </c>
     </row>
@@ -4794,7 +4794,7 @@
       <c r="M96" t="str">
         <v>LOW</v>
       </c>
-      <c r="P96" t="str">
+      <c r="N96" t="str">
         <v>N</v>
       </c>
     </row>
@@ -4838,7 +4838,7 @@
       <c r="M97" t="str">
         <v>LOW</v>
       </c>
-      <c r="P97" t="str">
+      <c r="N97" t="str">
         <v>N</v>
       </c>
     </row>
@@ -4882,7 +4882,7 @@
       <c r="M98" t="str">
         <v>LOW</v>
       </c>
-      <c r="P98" t="str">
+      <c r="N98" t="str">
         <v>N</v>
       </c>
     </row>
@@ -4924,13 +4924,13 @@
         <v>HIGH_RISK</v>
       </c>
       <c r="N99" t="str">
+        <v>Y</v>
+      </c>
+      <c r="O99" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O99" t="str">
+      <c r="P99" t="str">
         <v>ELECTRICAL_RISK</v>
-      </c>
-      <c r="P99" t="str">
-        <v>Y</v>
       </c>
     </row>
     <row r="100">
@@ -4971,13 +4971,13 @@
         <v>HIGH_RISK</v>
       </c>
       <c r="N100" t="str">
+        <v>Y</v>
+      </c>
+      <c r="O100" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O100" t="str">
+      <c r="P100" t="str">
         <v>ELECTRICAL_RISK</v>
-      </c>
-      <c r="P100" t="str">
-        <v>Y</v>
       </c>
     </row>
     <row r="101">
@@ -5021,13 +5021,13 @@
         <v>HIGH_RISK</v>
       </c>
       <c r="N101" t="str">
+        <v>Y</v>
+      </c>
+      <c r="O101" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O101" t="str">
+      <c r="P101" t="str">
         <v>PLUMBING_RISK</v>
-      </c>
-      <c r="P101" t="str">
-        <v>Y</v>
       </c>
     </row>
     <row r="102">
@@ -5071,13 +5071,13 @@
         <v>HIGH_RISK</v>
       </c>
       <c r="N102" t="str">
+        <v>Y</v>
+      </c>
+      <c r="O102" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O102" t="str">
+      <c r="P102" t="str">
         <v>PLUMBING_RISK</v>
-      </c>
-      <c r="P102" t="str">
-        <v>Y</v>
       </c>
     </row>
     <row r="103">
@@ -5120,11 +5120,11 @@
       <c r="M103" t="str">
         <v>LOW</v>
       </c>
-      <c r="O103" t="str">
+      <c r="N103" t="str">
+        <v>N</v>
+      </c>
+      <c r="P103" t="str">
         <v>ELECTRICAL_RISK</v>
-      </c>
-      <c r="P103" t="str">
-        <v>N</v>
       </c>
     </row>
     <row r="104">
@@ -5165,17 +5165,16 @@
         <v>HIGH_RISK</v>
       </c>
       <c r="N104" t="str">
+        <v>Y</v>
+      </c>
+      <c r="O104" t="str">
         <v>PER_ITEM_AFTER</v>
       </c>
-      <c r="O104" t="str">
+      <c r="P104" t="str">
         <v>ELECTRICAL_RISK</v>
       </c>
-      <c r="P104" t="str">
-        <v>Y</v>
-      </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:P104"/>
   </ignoredErrors>
@@ -18199,7 +18198,7 @@
         <v>60</v>
       </c>
       <c r="D5">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="E5" t="str">
         <v>(Synced from legacy columns Tier/Max_Hours/Customer_Price for parser compatibility.)</v>
@@ -18250,7 +18249,7 @@
         <v>60</v>
       </c>
       <c r="D8">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="E8" t="str">
         <v>(Synced from legacy columns Tier/Max_Hours/Customer_Price for parser compatibility.)</v>
@@ -18393,7 +18392,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:E16"/>
   </ignoredErrors>
@@ -19456,7 +19454,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D10"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -19519,10 +19517,10 @@
         <v>cable_concealment</v>
       </c>
       <c r="B5" t="str">
-        <v>cable,wire</v>
+        <v>cable</v>
       </c>
       <c r="C5" t="str">
-        <v>hide,conceal,cover,tidy,run,trunking</v>
+        <v>hide,conceal,cover,tidy,run,trunking,up,the,wires,some,cables,a</v>
       </c>
       <c r="D5" t="str">
         <v/>
@@ -19564,15 +19562,43 @@
         <v>hole</v>
       </c>
       <c r="C8" t="str">
-        <v>fill,patch,repair</v>
+        <v>fill,patch,repair,wall,in,the,a,holes</v>
       </c>
       <c r="D8" t="str">
         <v/>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>tap_leak_fix</v>
+      </c>
+      <c r="B9" t="str">
+        <v>tap</v>
+      </c>
+      <c r="C9" t="str">
+        <v>leak,fix,repair,drip,leaky,taps</v>
+      </c>
+      <c r="D9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>socket_replace</v>
+      </c>
+      <c r="B10" t="str">
+        <v>switch</v>
+      </c>
+      <c r="C10" t="str">
+        <v>replace,fix,change,install,light,sockets,socket,a</v>
+      </c>
+      <c r="D10" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D10"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>